<commit_message>
feat(lulu): Columbia v4.3.0 pilot — Sheet 15 Auto-Inferences + autoInferences JSON block
- Add Sheet 15 'Auto-Infer' to LULU Excel with 3 decision points (S&M Treatment, g_organic, b_growth), Phase 4 Audit Gate v4.3 result (PASS_WITH_ALERTS).
- Add autoInferences block to lulu.json with traceable confidence labels and fallback chains.
- Supabase company_dashboards row updated in parallel via jsonb_set so /api/dashboard reflects the new block immediately.
- Helpers live in skill columbia-valuation/helpers/: stable_regime_detector, sm_decision_point, historical_window_selector, audit_gate_v43, sector_fallback_table.
- LULU is the pilot for v4.3.0; MSFT/BKNG/SAP/RACE remain on v4.2.0 and will be recalibrated at next quarterly re-underwriting.

Refs: 5 CIO-ratified technical recommendations (28-may-2026).
🤖 Generated with Claude (Computer)
</commit_message>
<xml_diff>
--- a/public/docs/DCE_LULU_Columbia_Model.xlsx
+++ b/public/docs/DCE_LULU_Columbia_Model.xlsx
@@ -21,6 +21,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12. Implied IRR" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13. Summary" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14. Audit" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15. Auto-Infer" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -37,7 +38,7 @@
     <numFmt numFmtId="168" formatCode="0.0"/>
     <numFmt numFmtId="169" formatCode="+0.00%;-0.00%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -126,8 +127,49 @@
       <color rgb="FF008000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B2642"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00B88B47"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001B2642"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="001B2642"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00808080"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -164,6 +206,26 @@
         <bgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B2642"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00B88B47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E7D32"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F9A825"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -177,7 +239,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -355,6 +417,25 @@
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2760,7 +2841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="B2:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2770,7 +2851,6 @@
     <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="19" t="inlineStr">
         <is>
@@ -2785,7 +2865,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="5" t="inlineStr">
         <is>
@@ -2851,7 +2930,6 @@
         <v/>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="B12" s="5" t="inlineStr">
         <is>
@@ -2884,7 +2962,6 @@
         <v/>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="B16" s="5" t="inlineStr">
         <is>
@@ -2973,7 +3050,6 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
@@ -3071,7 +3147,6 @@
         <v/>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="B34" s="5" t="inlineStr">
         <is>
@@ -3125,7 +3200,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="B40" s="5" t="inlineStr">
         <is>
@@ -3189,7 +3263,6 @@
         <v/>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="B47" s="5" t="inlineStr">
         <is>
@@ -3265,7 +3338,6 @@
         <v/>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="B55" s="41" t="inlineStr">
         <is>
@@ -3295,7 +3367,6 @@
         <v/>
       </c>
     </row>
-    <row r="58"/>
     <row r="59">
       <c r="B59" s="28" t="inlineStr">
         <is>
@@ -3303,7 +3374,6 @@
         </is>
       </c>
     </row>
-    <row r="60"/>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="B3:E3"/>
@@ -4621,6 +4691,326 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B50:D50"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00B88B47"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:F34"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="72" t="inlineStr">
+        <is>
+          <t>SHEET 15 — AUTO-INFERENCES v4.3.0 | Lululemon Athletica Inc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="73" t="inlineStr">
+        <is>
+          <t>Layer de auto-inferencia trazable | Generado: 28-may-2026 | Helpers v4.3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="74" t="inlineStr">
+        <is>
+          <t>SM TREATMENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="75" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C6" s="76" t="inlineStr">
+        <is>
+          <t>Tier 2 — historical_ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="75" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="C7" s="82" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="75" t="inlineStr">
+        <is>
+          <t>Valor inferido</t>
+        </is>
+      </c>
+      <c r="C8" s="78" t="n">
+        <v>0.0333004123782791</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="75" t="inlineStr">
+        <is>
+          <t>Ventana histórica</t>
+        </is>
+      </c>
+      <c r="C9" s="76" t="inlineStr">
+        <is>
+          <t>Años: [2019, 2021, 2022, 2023, 2024, 2025] | Excluidos: [2020]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="75" t="inlineStr">
+        <is>
+          <t>Años estables</t>
+        </is>
+      </c>
+      <c r="C10" s="76" t="inlineStr">
+        <is>
+          <t>[2024, 2025]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="B11" s="75" t="inlineStr">
+        <is>
+          <t>Razonamiento</t>
+        </is>
+      </c>
+      <c r="C11" s="79" t="inlineStr">
+        <is>
+          <t>Baseline S&amp;M/Rev = 3.33% sobre 2 años estables. 2 stable years detected (growth band ±5.0pp, ratio band ±1.0pp). Median rev growth = 17.0%, median S&amp;M/Rev = 3.3%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="75" t="inlineStr">
+        <is>
+          <t>Fallback chain</t>
+        </is>
+      </c>
+      <c r="C12" s="79" t="inlineStr">
+        <is>
+          <t>Tier 1 (tano_pure) descartado: sin customer/churn data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="74" t="inlineStr">
+        <is>
+          <t>G ORGANIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="75" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C15" s="76" t="inlineStr">
+        <is>
+          <t>Tier 4 — manual_industry_long_run</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="75" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="C16" s="77" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="75" t="inlineStr">
+        <is>
+          <t>Valor inferido</t>
+        </is>
+      </c>
+      <c r="C17" s="78" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="B18" s="75" t="inlineStr">
+        <is>
+          <t>Razonamiento</t>
+        </is>
+      </c>
+      <c r="C18" s="79" t="inlineStr">
+        <is>
+          <t>US apparel industry long-run CAGR ≈ 3% (BEA + Statista 10y). LULU es consagrado, sin tailwind macro adicional. Tano method aplica el growth ex-empresa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="74" t="inlineStr">
+        <is>
+          <t>B GROWTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="75" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C21" s="76" t="inlineStr">
+        <is>
+          <t>Tier 2 — tano_capex_minus_da</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="75" t="inlineStr">
+        <is>
+          <t>Confidence</t>
+        </is>
+      </c>
+      <c r="C22" s="77" t="inlineStr">
+        <is>
+          <t>MEDIUM</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="75" t="inlineStr">
+        <is>
+          <t>Valor inferido</t>
+        </is>
+      </c>
+      <c r="C23" s="78" t="n">
+        <v>0.5891</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="75" t="inlineStr">
+        <is>
+          <t>Ventana histórica</t>
+        </is>
+      </c>
+      <c r="C24" s="76" t="inlineStr">
+        <is>
+          <t>Años: [2022, 2023, 2024, 2025] | Excluidos: [2020, 2021]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="50" customHeight="1">
+      <c r="B25" s="75" t="inlineStr">
+        <is>
+          <t>Razonamiento</t>
+        </is>
+      </c>
+      <c r="C25" s="79" t="inlineStr">
+        <is>
+          <t>Tano method: growth CapEx = Σ(CapEx) − Σ(D&amp;A) = 3047 − 1252 = 1795 sobre FY2022-2025. b_growth = 58.91%. Ventana 4y porque excluye FY2020-2021 (COVID disruption).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="74" t="inlineStr">
+        <is>
+          <t>PHASE 4 AUDIT GATE v4.3 — RESULTADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="75" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="C28" s="77" t="inlineStr">
+        <is>
+          <t>PASS_WITH_ALERTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="75" t="inlineStr">
+        <is>
+          <t>Confidence summary</t>
+        </is>
+      </c>
+      <c r="C29" s="76" t="inlineStr">
+        <is>
+          <t>HIGH=0  MEDIUM=2  LOW=1  FAIL=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="75" t="inlineStr">
+        <is>
+          <t>ROIC marginal</t>
+        </is>
+      </c>
+      <c r="C30" s="76" t="inlineStr">
+        <is>
+          <t>current=25.00%  previous=25.00%  Δ=+0bps</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="30" customHeight="1">
+      <c r="B31" s="75" t="inlineStr">
+        <is>
+          <t>Alerts</t>
+        </is>
+      </c>
+      <c r="C31" s="79" t="inlineStr">
+        <is>
+          <t>Phase 4 v4.3 Trigger A (sub-threshold): 1 LOW-confidence point(s): ['s&amp;m_treatment']. Below hard-fail threshold but flag for CIO review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="81" t="inlineStr">
+        <is>
+          <t>Generated by columbia-valuation v4.3.0 (helpers/) — DCE Holdings Confidential</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B34:F34"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="B27:F27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(lulu): dashboard v4.3.0 — IRR 47.73% + Probability tab (Bear 17.4% / Base 47.73% / Bull 47.71%) + autoInferences PASS_WITH_ALERTS
- Excel Sheet 12 row C37 g_organic 2% → 3% (v4.3.0 DP17 Tier 4 manual)
- Recálculo cascada: total growth 21.16% → 22.16%, IRR 46.61% → 47.73%, MoS 34.61pp → 35.73pp
- JSON irr.bearIrr=17.4 (Breaker), irr.bullIrr=47.71 (Builder v1.0), irr.bearDownside=-37.5
- JSON autoInferences re-injected con valueLabel correcto en cada DP
- thesisSummary.impliedIrr 46.61 → 47.73
- Narrative actualizada con buffer +35.73pp y Caso 2 marginal
</commit_message>
<xml_diff>
--- a/public/docs/DCE_LULU_Columbia_Model.xlsx
+++ b/public/docs/DCE_LULU_Columbia_Model.xlsx
@@ -3182,11 +3182,11 @@
     <row r="37">
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Crecimiento Orgánico (DP17)</t>
+          <t>Crecimiento Orgánico (DP17 — v4.3.0 Tier 4 manual)</t>
         </is>
       </c>
       <c r="C37" s="43" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="38">

</xml_diff>